<commit_message>
feat: encabezados descriptivos en resumen y tipo nombre en detalle
</commit_message>
<xml_diff>
--- a/Estimacion_Pruebas_Detallada.xlsx
+++ b/Estimacion_Pruebas_Detallada.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detalle de Casos" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Detalle de Casos'!$A$1:$G$109</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Detalle de Casos'!$A$1:$H$109</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -505,12 +505,12 @@
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="46" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="5" customWidth="1" min="5" max="5"/>
-    <col width="5" customWidth="1" min="6" max="6"/>
-    <col width="5" customWidth="1" min="7" max="7"/>
-    <col width="5" customWidth="1" min="8" max="8"/>
-    <col width="5" customWidth="1" min="9" max="9"/>
-    <col width="5" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
   </cols>
@@ -538,32 +538,32 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>Funcional</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>Datos / Reglas</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>Integración / API</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>Regresión</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>Visual / UI</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
@@ -1472,7 +1472,7 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>Datos/Reglas de negocio</t>
+          <t>Datos / Reglas de negocio</t>
         </is>
       </c>
       <c r="C3" s="10" t="n">
@@ -1487,7 +1487,7 @@
       </c>
       <c r="B4" s="10" t="inlineStr">
         <is>
-          <t>Integración/API</t>
+          <t>Integración / API</t>
         </is>
       </c>
       <c r="C4" s="10" t="n">
@@ -1532,7 +1532,7 @@
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>Visual/UI</t>
+          <t>Visual / UI</t>
         </is>
       </c>
       <c r="C7" s="10" t="n">
@@ -1550,7 +1550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G109"/>
+  <dimension ref="A1:H109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1559,7 +1559,8 @@
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="70" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1595,6 +1596,11 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Tipo (nombre)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Tiempo (min)</t>
         </is>
       </c>
@@ -1628,7 +1634,12 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G2" s="3" t="n">
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1661,7 +1672,12 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G3" s="6" t="n">
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1694,7 +1710,12 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G4" s="3" t="n">
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1727,7 +1748,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G5" s="6" t="n">
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="n">
         <v>20</v>
       </c>
     </row>
@@ -1760,7 +1786,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G6" s="3" t="n">
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="n">
         <v>20</v>
       </c>
     </row>
@@ -1793,7 +1824,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G7" s="6" t="n">
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="n">
         <v>20</v>
       </c>
     </row>
@@ -1826,7 +1862,12 @@
           <t>R</t>
         </is>
       </c>
-      <c r="G8" s="3" t="n">
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Regresión</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1859,7 +1900,12 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G9" s="6" t="n">
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1892,7 +1938,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G10" s="3" t="n">
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="n">
         <v>20</v>
       </c>
     </row>
@@ -1925,7 +1976,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G11" s="6" t="n">
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="n">
         <v>20</v>
       </c>
     </row>
@@ -1958,7 +2014,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G12" s="3" t="n">
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="n">
         <v>20</v>
       </c>
     </row>
@@ -1991,7 +2052,12 @@
           <t>R</t>
         </is>
       </c>
-      <c r="G13" s="6" t="n">
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Regresión</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="n">
         <v>15</v>
       </c>
     </row>
@@ -2024,7 +2090,12 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G14" s="3" t="n">
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="n">
         <v>15</v>
       </c>
     </row>
@@ -2057,7 +2128,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G15" s="6" t="n">
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2090,7 +2166,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G16" s="3" t="n">
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2123,7 +2204,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G17" s="6" t="n">
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2156,7 +2242,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G18" s="3" t="n">
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2189,7 +2280,12 @@
           <t>R</t>
         </is>
       </c>
-      <c r="G19" s="6" t="n">
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>Regresión</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="n">
         <v>15</v>
       </c>
     </row>
@@ -2222,7 +2318,12 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G20" s="3" t="n">
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="n">
         <v>15</v>
       </c>
     </row>
@@ -2255,7 +2356,12 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G21" s="6" t="n">
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="n">
         <v>15</v>
       </c>
     </row>
@@ -2288,7 +2394,12 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G22" s="3" t="n">
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="n">
         <v>15</v>
       </c>
     </row>
@@ -2321,7 +2432,12 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G23" s="6" t="n">
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="n">
         <v>15</v>
       </c>
     </row>
@@ -2354,7 +2470,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G24" s="3" t="n">
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2387,7 +2508,12 @@
           <t>R</t>
         </is>
       </c>
-      <c r="G25" s="6" t="n">
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>Regresión</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="n">
         <v>15</v>
       </c>
     </row>
@@ -2420,7 +2546,12 @@
           <t>V</t>
         </is>
       </c>
-      <c r="G26" s="3" t="n">
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -2453,7 +2584,12 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G27" s="6" t="n">
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="n">
         <v>15</v>
       </c>
     </row>
@@ -2486,7 +2622,12 @@
           <t>R</t>
         </is>
       </c>
-      <c r="G28" s="3" t="n">
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>Regresión</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="n">
         <v>15</v>
       </c>
     </row>
@@ -2519,7 +2660,12 @@
           <t>V</t>
         </is>
       </c>
-      <c r="G29" s="6" t="n">
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="H29" s="6" t="n">
         <v>10</v>
       </c>
     </row>
@@ -2552,7 +2698,12 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G30" s="3" t="n">
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="n">
         <v>15</v>
       </c>
     </row>
@@ -2585,7 +2736,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G31" s="6" t="n">
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2618,7 +2774,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G32" s="3" t="n">
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2651,7 +2812,12 @@
           <t>R</t>
         </is>
       </c>
-      <c r="G33" s="6" t="n">
+      <c r="G33" s="6" t="inlineStr">
+        <is>
+          <t>Regresión</t>
+        </is>
+      </c>
+      <c r="H33" s="6" t="n">
         <v>15</v>
       </c>
     </row>
@@ -2684,7 +2850,12 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G34" s="3" t="n">
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="n">
         <v>15</v>
       </c>
     </row>
@@ -2717,7 +2888,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G35" s="6" t="n">
+      <c r="G35" s="6" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H35" s="6" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2750,7 +2926,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G36" s="3" t="n">
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2783,7 +2964,12 @@
           <t>R</t>
         </is>
       </c>
-      <c r="G37" s="6" t="n">
+      <c r="G37" s="6" t="inlineStr">
+        <is>
+          <t>Regresión</t>
+        </is>
+      </c>
+      <c r="H37" s="6" t="n">
         <v>15</v>
       </c>
     </row>
@@ -2816,7 +3002,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G38" s="3" t="n">
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2849,7 +3040,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G39" s="6" t="n">
+      <c r="G39" s="6" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H39" s="6" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2882,7 +3078,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G40" s="3" t="n">
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2915,7 +3116,12 @@
           <t>R</t>
         </is>
       </c>
-      <c r="G41" s="6" t="n">
+      <c r="G41" s="6" t="inlineStr">
+        <is>
+          <t>Regresión</t>
+        </is>
+      </c>
+      <c r="H41" s="6" t="n">
         <v>15</v>
       </c>
     </row>
@@ -2948,7 +3154,12 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G42" s="3" t="n">
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="n">
         <v>15</v>
       </c>
     </row>
@@ -2981,7 +3192,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G43" s="6" t="n">
+      <c r="G43" s="6" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H43" s="6" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3014,7 +3230,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G44" s="3" t="n">
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3047,7 +3268,12 @@
           <t>R</t>
         </is>
       </c>
-      <c r="G45" s="6" t="n">
+      <c r="G45" s="6" t="inlineStr">
+        <is>
+          <t>Regresión</t>
+        </is>
+      </c>
+      <c r="H45" s="6" t="n">
         <v>15</v>
       </c>
     </row>
@@ -3080,7 +3306,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G46" s="3" t="n">
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3113,7 +3344,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G47" s="6" t="n">
+      <c r="G47" s="6" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H47" s="6" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3146,7 +3382,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G48" s="3" t="n">
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3179,7 +3420,12 @@
           <t>R</t>
         </is>
       </c>
-      <c r="G49" s="6" t="n">
+      <c r="G49" s="6" t="inlineStr">
+        <is>
+          <t>Regresión</t>
+        </is>
+      </c>
+      <c r="H49" s="6" t="n">
         <v>15</v>
       </c>
     </row>
@@ -3212,7 +3458,12 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G50" s="3" t="n">
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="n">
         <v>15</v>
       </c>
     </row>
@@ -3245,7 +3496,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G51" s="6" t="n">
+      <c r="G51" s="6" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H51" s="6" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3278,7 +3534,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G52" s="3" t="n">
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3311,7 +3572,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G53" s="6" t="n">
+      <c r="G53" s="6" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H53" s="6" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3344,7 +3610,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G54" s="3" t="n">
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3377,7 +3648,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G55" s="6" t="n">
+      <c r="G55" s="6" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H55" s="6" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3410,7 +3686,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G56" s="3" t="n">
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3443,7 +3724,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="G57" s="6" t="n">
+      <c r="G57" s="6" t="inlineStr">
+        <is>
+          <t>Integración</t>
+        </is>
+      </c>
+      <c r="H57" s="6" t="n">
         <v>25</v>
       </c>
     </row>
@@ -3476,7 +3762,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="G58" s="3" t="n">
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>Integración</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="n">
         <v>25</v>
       </c>
     </row>
@@ -3509,7 +3800,12 @@
           <t>S</t>
         </is>
       </c>
-      <c r="G59" s="6" t="n">
+      <c r="G59" s="6" t="inlineStr">
+        <is>
+          <t>Seguridad</t>
+        </is>
+      </c>
+      <c r="H59" s="6" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3542,7 +3838,12 @@
           <t>R</t>
         </is>
       </c>
-      <c r="G60" s="3" t="n">
+      <c r="G60" s="3" t="inlineStr">
+        <is>
+          <t>Regresión</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="n">
         <v>15</v>
       </c>
     </row>
@@ -3575,7 +3876,12 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G61" s="6" t="n">
+      <c r="G61" s="6" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="H61" s="6" t="n">
         <v>15</v>
       </c>
     </row>
@@ -3608,7 +3914,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G62" s="3" t="n">
+      <c r="G62" s="3" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H62" s="3" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3641,7 +3952,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G63" s="6" t="n">
+      <c r="G63" s="6" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H63" s="6" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3674,7 +3990,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G64" s="3" t="n">
+      <c r="G64" s="3" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3707,7 +4028,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G65" s="6" t="n">
+      <c r="G65" s="6" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H65" s="6" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3740,7 +4066,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G66" s="3" t="n">
+      <c r="G66" s="3" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H66" s="3" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3773,7 +4104,12 @@
           <t>R</t>
         </is>
       </c>
-      <c r="G67" s="6" t="n">
+      <c r="G67" s="6" t="inlineStr">
+        <is>
+          <t>Regresión</t>
+        </is>
+      </c>
+      <c r="H67" s="6" t="n">
         <v>15</v>
       </c>
     </row>
@@ -3806,7 +4142,12 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G68" s="3" t="n">
+      <c r="G68" s="3" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="H68" s="3" t="n">
         <v>15</v>
       </c>
     </row>
@@ -3839,7 +4180,12 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G69" s="6" t="n">
+      <c r="G69" s="6" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="H69" s="6" t="n">
         <v>15</v>
       </c>
     </row>
@@ -3872,7 +4218,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G70" s="3" t="n">
+      <c r="G70" s="3" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H70" s="3" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3905,7 +4256,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G71" s="6" t="n">
+      <c r="G71" s="6" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H71" s="6" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3938,7 +4294,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G72" s="3" t="n">
+      <c r="G72" s="3" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H72" s="3" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3971,7 +4332,12 @@
           <t>R</t>
         </is>
       </c>
-      <c r="G73" s="6" t="n">
+      <c r="G73" s="6" t="inlineStr">
+        <is>
+          <t>Regresión</t>
+        </is>
+      </c>
+      <c r="H73" s="6" t="n">
         <v>15</v>
       </c>
     </row>
@@ -4004,7 +4370,12 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G74" s="3" t="n">
+      <c r="G74" s="3" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="H74" s="3" t="n">
         <v>15</v>
       </c>
     </row>
@@ -4037,7 +4408,12 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G75" s="6" t="n">
+      <c r="G75" s="6" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="H75" s="6" t="n">
         <v>15</v>
       </c>
     </row>
@@ -4070,7 +4446,12 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G76" s="3" t="n">
+      <c r="G76" s="3" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="H76" s="3" t="n">
         <v>15</v>
       </c>
     </row>
@@ -4103,7 +4484,12 @@
           <t>S</t>
         </is>
       </c>
-      <c r="G77" s="6" t="n">
+      <c r="G77" s="6" t="inlineStr">
+        <is>
+          <t>Seguridad</t>
+        </is>
+      </c>
+      <c r="H77" s="6" t="n">
         <v>20</v>
       </c>
     </row>
@@ -4136,7 +4522,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G78" s="3" t="n">
+      <c r="G78" s="3" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H78" s="3" t="n">
         <v>20</v>
       </c>
     </row>
@@ -4169,7 +4560,12 @@
           <t>R</t>
         </is>
       </c>
-      <c r="G79" s="6" t="n">
+      <c r="G79" s="6" t="inlineStr">
+        <is>
+          <t>Regresión</t>
+        </is>
+      </c>
+      <c r="H79" s="6" t="n">
         <v>15</v>
       </c>
     </row>
@@ -4202,7 +4598,12 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G80" s="3" t="n">
+      <c r="G80" s="3" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="H80" s="3" t="n">
         <v>15</v>
       </c>
     </row>
@@ -4235,7 +4636,12 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G81" s="6" t="n">
+      <c r="G81" s="6" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="H81" s="6" t="n">
         <v>15</v>
       </c>
     </row>
@@ -4268,7 +4674,12 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G82" s="3" t="n">
+      <c r="G82" s="3" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="H82" s="3" t="n">
         <v>15</v>
       </c>
     </row>
@@ -4301,7 +4712,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="G83" s="6" t="n">
+      <c r="G83" s="6" t="inlineStr">
+        <is>
+          <t>Integración</t>
+        </is>
+      </c>
+      <c r="H83" s="6" t="n">
         <v>25</v>
       </c>
     </row>
@@ -4334,7 +4750,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="G84" s="3" t="n">
+      <c r="G84" s="3" t="inlineStr">
+        <is>
+          <t>Integración</t>
+        </is>
+      </c>
+      <c r="H84" s="3" t="n">
         <v>25</v>
       </c>
     </row>
@@ -4367,7 +4788,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G85" s="6" t="n">
+      <c r="G85" s="6" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H85" s="6" t="n">
         <v>20</v>
       </c>
     </row>
@@ -4400,7 +4826,12 @@
           <t>R</t>
         </is>
       </c>
-      <c r="G86" s="3" t="n">
+      <c r="G86" s="3" t="inlineStr">
+        <is>
+          <t>Regresión</t>
+        </is>
+      </c>
+      <c r="H86" s="3" t="n">
         <v>15</v>
       </c>
     </row>
@@ -4433,7 +4864,12 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G87" s="6" t="n">
+      <c r="G87" s="6" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="H87" s="6" t="n">
         <v>15</v>
       </c>
     </row>
@@ -4466,7 +4902,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G88" s="3" t="n">
+      <c r="G88" s="3" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H88" s="3" t="n">
         <v>20</v>
       </c>
     </row>
@@ -4499,7 +4940,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G89" s="6" t="n">
+      <c r="G89" s="6" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H89" s="6" t="n">
         <v>20</v>
       </c>
     </row>
@@ -4532,7 +4978,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G90" s="3" t="n">
+      <c r="G90" s="3" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H90" s="3" t="n">
         <v>20</v>
       </c>
     </row>
@@ -4565,7 +5016,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G91" s="6" t="n">
+      <c r="G91" s="6" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H91" s="6" t="n">
         <v>20</v>
       </c>
     </row>
@@ -4598,7 +5054,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G92" s="3" t="n">
+      <c r="G92" s="3" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H92" s="3" t="n">
         <v>20</v>
       </c>
     </row>
@@ -4631,7 +5092,12 @@
           <t>R</t>
         </is>
       </c>
-      <c r="G93" s="6" t="n">
+      <c r="G93" s="6" t="inlineStr">
+        <is>
+          <t>Regresión</t>
+        </is>
+      </c>
+      <c r="H93" s="6" t="n">
         <v>15</v>
       </c>
     </row>
@@ -4664,7 +5130,12 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G94" s="3" t="n">
+      <c r="G94" s="3" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="H94" s="3" t="n">
         <v>15</v>
       </c>
     </row>
@@ -4697,7 +5168,12 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G95" s="6" t="n">
+      <c r="G95" s="6" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="H95" s="6" t="n">
         <v>15</v>
       </c>
     </row>
@@ -4730,7 +5206,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G96" s="3" t="n">
+      <c r="G96" s="3" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H96" s="3" t="n">
         <v>20</v>
       </c>
     </row>
@@ -4763,7 +5244,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G97" s="6" t="n">
+      <c r="G97" s="6" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H97" s="6" t="n">
         <v>20</v>
       </c>
     </row>
@@ -4796,7 +5282,12 @@
           <t>R</t>
         </is>
       </c>
-      <c r="G98" s="3" t="n">
+      <c r="G98" s="3" t="inlineStr">
+        <is>
+          <t>Regresión</t>
+        </is>
+      </c>
+      <c r="H98" s="3" t="n">
         <v>15</v>
       </c>
     </row>
@@ -4829,7 +5320,12 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G99" s="6" t="n">
+      <c r="G99" s="6" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="H99" s="6" t="n">
         <v>15</v>
       </c>
     </row>
@@ -4862,7 +5358,12 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G100" s="3" t="n">
+      <c r="G100" s="3" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="H100" s="3" t="n">
         <v>15</v>
       </c>
     </row>
@@ -4895,7 +5396,12 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G101" s="6" t="n">
+      <c r="G101" s="6" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="H101" s="6" t="n">
         <v>15</v>
       </c>
     </row>
@@ -4928,7 +5434,12 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G102" s="3" t="n">
+      <c r="G102" s="3" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="H102" s="3" t="n">
         <v>15</v>
       </c>
     </row>
@@ -4961,7 +5472,12 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G103" s="6" t="n">
+      <c r="G103" s="6" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="H103" s="6" t="n">
         <v>15</v>
       </c>
     </row>
@@ -4994,7 +5510,12 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G104" s="3" t="n">
+      <c r="G104" s="3" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="H104" s="3" t="n">
         <v>15</v>
       </c>
     </row>
@@ -5027,7 +5548,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="G105" s="6" t="n">
+      <c r="G105" s="6" t="inlineStr">
+        <is>
+          <t>Integración</t>
+        </is>
+      </c>
+      <c r="H105" s="6" t="n">
         <v>25</v>
       </c>
     </row>
@@ -5060,7 +5586,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G106" s="3" t="n">
+      <c r="G106" s="3" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H106" s="3" t="n">
         <v>20</v>
       </c>
     </row>
@@ -5093,7 +5624,12 @@
           <t>D</t>
         </is>
       </c>
-      <c r="G107" s="6" t="n">
+      <c r="G107" s="6" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="H107" s="6" t="n">
         <v>20</v>
       </c>
     </row>
@@ -5126,7 +5662,12 @@
           <t>S</t>
         </is>
       </c>
-      <c r="G108" s="3" t="n">
+      <c r="G108" s="3" t="inlineStr">
+        <is>
+          <t>Seguridad</t>
+        </is>
+      </c>
+      <c r="H108" s="3" t="n">
         <v>20</v>
       </c>
     </row>
@@ -5159,12 +5700,17 @@
           <t>R</t>
         </is>
       </c>
-      <c r="G109" s="6" t="n">
+      <c r="G109" s="6" t="inlineStr">
+        <is>
+          <t>Regresión</t>
+        </is>
+      </c>
+      <c r="H109" s="6" t="n">
         <v>15</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G109"/>
+  <autoFilter ref="A1:H109"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>